<commit_message>
add migrationBackground to PupilIdentity, update excel template
</commit_message>
<xml_diff>
--- a/test_data/schild_export_excel_template.xlsx
+++ b/test_data/schild_export_excel_template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\code\dabblingwithcode\school_data_hub\test_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F8FF753-E2E0-4530-B64C-24918BB3F95D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{40B7D391-08F3-41BF-B0B6-641CA7FE0B97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="29535" yWindow="2880" windowWidth="21600" windowHeight="7890" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Datenexport" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
   <si>
     <t>Interne ID-Nummer</t>
   </si>
@@ -55,6 +55,9 @@
     <t>Staatsangehörigkeit (Schlüssel)</t>
   </si>
   <si>
+    <t>Migrationshintergrund vorhanden</t>
+  </si>
+  <si>
     <t>Verkehrssprache in der Familie</t>
   </si>
   <si>
@@ -89,48 +92,6 @@
   </si>
   <si>
     <t>Entlassdatum</t>
-  </si>
-  <si>
-    <t>A1</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>04</t>
-  </si>
-  <si>
-    <t>LE</t>
-  </si>
-  <si>
-    <t>w</t>
-  </si>
-  <si>
-    <t>000</t>
-  </si>
-  <si>
-    <t>Türkisch</t>
-  </si>
-  <si>
-    <t>2021-08-01</t>
-  </si>
-  <si>
-    <t>OFFGANZ</t>
-  </si>
-  <si>
-    <t>isl.</t>
-  </si>
-  <si>
-    <t>2024-08-28</t>
-  </si>
-  <si>
-    <t>Fake</t>
-  </si>
-  <si>
-    <t>Lastname</t>
-  </si>
-  <si>
-    <t>BUW</t>
   </si>
 </sst>
 </file>
@@ -159,7 +120,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -167,42 +128,13 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color theme="9" tint="0.39997558519241921"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color theme="9" tint="0.39997558519241921"/>
-      </top>
-      <bottom style="thin">
-        <color theme="9" tint="0.39997558519241921"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color theme="9" tint="0.39997558519241921"/>
-      </right>
-      <top style="thin">
-        <color theme="9" tint="0.39997558519241921"/>
-      </top>
-      <bottom style="thin">
-        <color theme="9" tint="0.39997558519241921"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="1" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
@@ -508,32 +440,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:W2"/>
+  <dimension ref="A1:X1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="19.5703125" customWidth="1"/>
-    <col min="2" max="2" width="10.28515625" customWidth="1"/>
-    <col min="5" max="5" width="19.85546875" customWidth="1"/>
-    <col min="6" max="6" width="24" customWidth="1"/>
-    <col min="7" max="7" width="9.42578125" customWidth="1"/>
-    <col min="8" max="8" width="21.140625" customWidth="1"/>
-    <col min="9" max="9" width="21" customWidth="1"/>
-    <col min="11" max="11" width="28.7109375" customWidth="1"/>
-    <col min="12" max="12" width="29.140625" customWidth="1"/>
-    <col min="13" max="13" width="21.85546875" customWidth="1"/>
-    <col min="14" max="14" width="17" customWidth="1"/>
-    <col min="15" max="15" width="29.42578125" customWidth="1"/>
-    <col min="16" max="16" width="18.28515625" customWidth="1"/>
-    <col min="17" max="17" width="16" customWidth="1"/>
-    <col min="18" max="18" width="20.42578125" customWidth="1"/>
-    <col min="19" max="19" width="19.7109375" customWidth="1"/>
-    <col min="20" max="20" width="20.42578125" customWidth="1"/>
-    <col min="21" max="21" width="17" customWidth="1"/>
-    <col min="22" max="22" width="21.85546875" customWidth="1"/>
-    <col min="23" max="23" width="15.140625" customWidth="1"/>
-  </cols>
   <sheetData>
-    <row r="1" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -603,76 +513,8 @@
       <c r="W1" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="2" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A2">
-        <v>9862</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="D2" t="s">
+      <c r="X1" t="s">
         <v>23</v>
-      </c>
-      <c r="E2" t="s">
-        <v>36</v>
-      </c>
-      <c r="F2" t="s">
-        <v>24</v>
-      </c>
-      <c r="G2" t="s">
-        <v>25</v>
-      </c>
-      <c r="H2" t="s">
-        <v>26</v>
-      </c>
-      <c r="I2" t="s">
-        <v>24</v>
-      </c>
-      <c r="J2" t="s">
-        <v>27</v>
-      </c>
-      <c r="K2" t="s">
-        <v>28</v>
-      </c>
-      <c r="L2" t="s">
-        <v>29</v>
-      </c>
-      <c r="M2" t="s">
-        <v>24</v>
-      </c>
-      <c r="N2" s="3">
-        <v>42013</v>
-      </c>
-      <c r="O2" t="s">
-        <v>24</v>
-      </c>
-      <c r="P2" t="s">
-        <v>30</v>
-      </c>
-      <c r="Q2" t="s">
-        <v>31</v>
-      </c>
-      <c r="R2" t="s">
-        <v>32</v>
-      </c>
-      <c r="S2" t="s">
-        <v>33</v>
-      </c>
-      <c r="T2" t="s">
-        <v>24</v>
-      </c>
-      <c r="U2" t="s">
-        <v>24</v>
-      </c>
-      <c r="V2" t="s">
-        <v>24</v>
-      </c>
-      <c r="W2" t="s">
-        <v>24</v>
       </c>
     </row>
   </sheetData>

</xml_diff>